<commit_message>
Use fast greedy solver in web API and commit deduped course data + solved outputs
- web/main.py: solve endpoint now uses fast_solver.greedy_phase1 (fast_solver.py)
  instead of CP-SAT; both semesters solve in ~35s/25s with zero conflicts
  and 97-100% utilization.
- courses.xlsx (sem1/sem2): deduped and relinked (cross-programme groups,
  split same-programme A/B sections) so population never exceeds 120-cap rooms.
- output: regenerated zero-conflict timetables and timetable_rows for both semesters.
- Add fast_solver.py as runtime dependency of the web solve path.
- gitignore: ignore .admin_credentials (admin secret).
</commit_message>
<xml_diff>
--- a/data/semesters/sem2/courses.xlsx
+++ b/data/semesters/sem2/courses.xlsx
@@ -1804,11 +1804,7 @@
       <c r="Q21" t="n">
         <v>119</v>
       </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>joint-20</t>
-        </is>
-      </c>
+      <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1873,11 +1869,7 @@
       <c r="Q22" t="n">
         <v>15</v>
       </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>joint-20</t>
-        </is>
-      </c>
+      <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -4719,11 +4711,7 @@
       <c r="Q66" t="n">
         <v>119</v>
       </c>
-      <c r="R66" t="inlineStr">
-        <is>
-          <t>joint-64</t>
-        </is>
-      </c>
+      <c r="R66" t="inlineStr"/>
       <c r="S66" t="inlineStr"/>
     </row>
     <row r="67">
@@ -4792,11 +4780,7 @@
       <c r="Q67" t="n">
         <v>116</v>
       </c>
-      <c r="R67" t="inlineStr">
-        <is>
-          <t>joint-64</t>
-        </is>
-      </c>
+      <c r="R67" t="inlineStr"/>
       <c r="S67" t="inlineStr"/>
     </row>
     <row r="68">
@@ -12121,11 +12105,7 @@
       <c r="Q180" t="n">
         <v>120</v>
       </c>
-      <c r="R180" t="inlineStr">
-        <is>
-          <t>joint-175</t>
-        </is>
-      </c>
+      <c r="R180" t="inlineStr"/>
       <c r="S180" t="inlineStr"/>
     </row>
     <row r="181">
@@ -12194,11 +12174,7 @@
       <c r="Q181" t="n">
         <v>25</v>
       </c>
-      <c r="R181" t="inlineStr">
-        <is>
-          <t>joint-175</t>
-        </is>
-      </c>
+      <c r="R181" t="inlineStr"/>
       <c r="S181" t="inlineStr"/>
     </row>
     <row r="182">
@@ -18392,11 +18368,7 @@
       <c r="Q277" t="n">
         <v>112</v>
       </c>
-      <c r="R277" t="inlineStr">
-        <is>
-          <t>joint-271</t>
-        </is>
-      </c>
+      <c r="R277" t="inlineStr"/>
       <c r="S277" t="inlineStr"/>
     </row>
     <row r="278">
@@ -18465,11 +18437,7 @@
       <c r="Q278" t="n">
         <v>116</v>
       </c>
-      <c r="R278" t="inlineStr">
-        <is>
-          <t>joint-271</t>
-        </is>
-      </c>
+      <c r="R278" t="inlineStr"/>
       <c r="S278" t="inlineStr"/>
     </row>
     <row r="279">
@@ -19562,11 +19530,7 @@
       <c r="Q295" t="n">
         <v>112</v>
       </c>
-      <c r="R295" t="inlineStr">
-        <is>
-          <t>joint-288</t>
-        </is>
-      </c>
+      <c r="R295" t="inlineStr"/>
       <c r="S295" t="inlineStr"/>
     </row>
     <row r="296">
@@ -19635,11 +19599,7 @@
       <c r="Q296" t="n">
         <v>112</v>
       </c>
-      <c r="R296" t="inlineStr">
-        <is>
-          <t>joint-288</t>
-        </is>
-      </c>
+      <c r="R296" t="inlineStr"/>
       <c r="S296" t="inlineStr"/>
     </row>
     <row r="297">
@@ -19708,11 +19668,7 @@
       <c r="Q297" t="n">
         <v>116</v>
       </c>
-      <c r="R297" t="inlineStr">
-        <is>
-          <t>joint-288</t>
-        </is>
-      </c>
+      <c r="R297" t="inlineStr"/>
       <c r="S297" t="inlineStr"/>
     </row>
     <row r="298">
@@ -24094,11 +24050,7 @@
       <c r="Q365" t="n">
         <v>112</v>
       </c>
-      <c r="R365" t="inlineStr">
-        <is>
-          <t>joint-356</t>
-        </is>
-      </c>
+      <c r="R365" t="inlineStr"/>
       <c r="S365" t="inlineStr"/>
     </row>
     <row r="366">
@@ -24167,11 +24119,7 @@
       <c r="Q366" t="n">
         <v>119</v>
       </c>
-      <c r="R366" t="inlineStr">
-        <is>
-          <t>joint-356</t>
-        </is>
-      </c>
+      <c r="R366" t="inlineStr"/>
       <c r="S366" t="inlineStr"/>
     </row>
     <row r="367">
@@ -26696,11 +26644,7 @@
       <c r="Q405" t="n">
         <v>116</v>
       </c>
-      <c r="R405" t="inlineStr">
-        <is>
-          <t>joint-395</t>
-        </is>
-      </c>
+      <c r="R405" t="inlineStr"/>
       <c r="S405" t="inlineStr"/>
     </row>
     <row r="406">
@@ -26769,11 +26713,7 @@
       <c r="Q406" t="n">
         <v>116</v>
       </c>
-      <c r="R406" t="inlineStr">
-        <is>
-          <t>joint-395</t>
-        </is>
-      </c>
+      <c r="R406" t="inlineStr"/>
       <c r="S406" t="inlineStr"/>
     </row>
     <row r="407">
@@ -26842,11 +26782,7 @@
       <c r="Q407" t="n">
         <v>112</v>
       </c>
-      <c r="R407" t="inlineStr">
-        <is>
-          <t>joint-395</t>
-        </is>
-      </c>
+      <c r="R407" t="inlineStr"/>
       <c r="S407" t="inlineStr"/>
     </row>
     <row r="408">
@@ -28579,11 +28515,7 @@
       <c r="Q434" t="n">
         <v>116</v>
       </c>
-      <c r="R434" t="inlineStr">
-        <is>
-          <t>joint-422</t>
-        </is>
-      </c>
+      <c r="R434" t="inlineStr"/>
       <c r="S434" t="inlineStr"/>
     </row>
     <row r="435">
@@ -28652,11 +28584,7 @@
       <c r="Q435" t="n">
         <v>112</v>
       </c>
-      <c r="R435" t="inlineStr">
-        <is>
-          <t>joint-422</t>
-        </is>
-      </c>
+      <c r="R435" t="inlineStr"/>
       <c r="S435" t="inlineStr"/>
     </row>
     <row r="436">
@@ -28725,11 +28653,7 @@
       <c r="Q436" t="n">
         <v>112</v>
       </c>
-      <c r="R436" t="inlineStr">
-        <is>
-          <t>joint-422</t>
-        </is>
-      </c>
+      <c r="R436" t="inlineStr"/>
       <c r="S436" t="inlineStr"/>
     </row>
     <row r="437">
@@ -28798,11 +28722,7 @@
       <c r="Q437" t="n">
         <v>116</v>
       </c>
-      <c r="R437" t="inlineStr">
-        <is>
-          <t>joint-423</t>
-        </is>
-      </c>
+      <c r="R437" t="inlineStr"/>
       <c r="S437" t="inlineStr"/>
     </row>
     <row r="438">
@@ -28871,11 +28791,7 @@
       <c r="Q438" t="n">
         <v>112</v>
       </c>
-      <c r="R438" t="inlineStr">
-        <is>
-          <t>joint-423</t>
-        </is>
-      </c>
+      <c r="R438" t="inlineStr"/>
       <c r="S438" t="inlineStr"/>
     </row>
     <row r="439">
@@ -29858,14 +29774,8 @@
       <c r="Q453" t="n">
         <v>117</v>
       </c>
-      <c r="R453" t="inlineStr">
-        <is>
-          <t>joint-437</t>
-        </is>
-      </c>
-      <c r="S453" t="n">
-        <v>120</v>
-      </c>
+      <c r="R453" t="inlineStr"/>
+      <c r="S453" t="inlineStr"/>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
@@ -29929,14 +29839,8 @@
       <c r="Q454" t="n">
         <v>15</v>
       </c>
-      <c r="R454" t="inlineStr">
-        <is>
-          <t>joint-437</t>
-        </is>
-      </c>
-      <c r="S454" t="n">
-        <v>120</v>
-      </c>
+      <c r="R454" t="inlineStr"/>
+      <c r="S454" t="inlineStr"/>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -33181,11 +33085,7 @@
       <c r="Q504" t="n">
         <v>117</v>
       </c>
-      <c r="R504" t="inlineStr">
-        <is>
-          <t>joint-487</t>
-        </is>
-      </c>
+      <c r="R504" t="inlineStr"/>
       <c r="S504" t="inlineStr"/>
     </row>
     <row r="505">
@@ -33254,11 +33154,7 @@
       <c r="Q505" t="n">
         <v>120</v>
       </c>
-      <c r="R505" t="inlineStr">
-        <is>
-          <t>joint-487</t>
-        </is>
-      </c>
+      <c r="R505" t="inlineStr"/>
       <c r="S505" t="inlineStr"/>
     </row>
     <row r="506">
@@ -33969,11 +33865,7 @@
       <c r="Q516" t="n">
         <v>117</v>
       </c>
-      <c r="R516" t="inlineStr">
-        <is>
-          <t>joint-498</t>
-        </is>
-      </c>
+      <c r="R516" t="inlineStr"/>
       <c r="S516" t="inlineStr"/>
     </row>
     <row r="517">
@@ -34042,11 +33934,7 @@
       <c r="Q517" t="n">
         <v>119</v>
       </c>
-      <c r="R517" t="inlineStr">
-        <is>
-          <t>joint-498</t>
-        </is>
-      </c>
+      <c r="R517" t="inlineStr"/>
       <c r="S517" t="inlineStr"/>
     </row>
     <row r="518">
@@ -34115,11 +34003,7 @@
       <c r="Q518" t="n">
         <v>120</v>
       </c>
-      <c r="R518" t="inlineStr">
-        <is>
-          <t>joint-498</t>
-        </is>
-      </c>
+      <c r="R518" t="inlineStr"/>
       <c r="S518" t="inlineStr"/>
     </row>
     <row r="519">
@@ -34188,11 +34072,7 @@
       <c r="Q519" t="n">
         <v>40</v>
       </c>
-      <c r="R519" t="inlineStr">
-        <is>
-          <t>joint-498</t>
-        </is>
-      </c>
+      <c r="R519" t="inlineStr"/>
       <c r="S519" t="inlineStr"/>
     </row>
     <row r="520">
@@ -34261,11 +34141,7 @@
       <c r="Q520" t="n">
         <v>117</v>
       </c>
-      <c r="R520" t="inlineStr">
-        <is>
-          <t>joint-499</t>
-        </is>
-      </c>
+      <c r="R520" t="inlineStr"/>
       <c r="S520" t="inlineStr"/>
     </row>
     <row r="521">
@@ -34334,11 +34210,7 @@
       <c r="Q521" t="n">
         <v>40</v>
       </c>
-      <c r="R521" t="inlineStr">
-        <is>
-          <t>joint-499</t>
-        </is>
-      </c>
+      <c r="R521" t="inlineStr"/>
       <c r="S521" t="inlineStr"/>
     </row>
     <row r="522">
@@ -34407,11 +34279,7 @@
       <c r="Q522" t="n">
         <v>117</v>
       </c>
-      <c r="R522" t="inlineStr">
-        <is>
-          <t>joint-500</t>
-        </is>
-      </c>
+      <c r="R522" t="inlineStr"/>
       <c r="S522" t="inlineStr"/>
     </row>
     <row r="523">
@@ -34480,11 +34348,7 @@
       <c r="Q523" t="n">
         <v>120</v>
       </c>
-      <c r="R523" t="inlineStr">
-        <is>
-          <t>joint-500</t>
-        </is>
-      </c>
+      <c r="R523" t="inlineStr"/>
       <c r="S523" t="inlineStr"/>
     </row>
     <row r="524">
@@ -34553,11 +34417,7 @@
       <c r="Q524" t="n">
         <v>117</v>
       </c>
-      <c r="R524" t="inlineStr">
-        <is>
-          <t>joint-501</t>
-        </is>
-      </c>
+      <c r="R524" t="inlineStr"/>
       <c r="S524" t="inlineStr"/>
     </row>
     <row r="525">
@@ -34626,11 +34486,7 @@
       <c r="Q525" t="n">
         <v>120</v>
       </c>
-      <c r="R525" t="inlineStr">
-        <is>
-          <t>joint-501</t>
-        </is>
-      </c>
+      <c r="R525" t="inlineStr"/>
       <c r="S525" t="inlineStr"/>
     </row>
     <row r="526">
@@ -34699,11 +34555,7 @@
       <c r="Q526" t="n">
         <v>40</v>
       </c>
-      <c r="R526" t="inlineStr">
-        <is>
-          <t>joint-501</t>
-        </is>
-      </c>
+      <c r="R526" t="inlineStr"/>
       <c r="S526" t="inlineStr"/>
     </row>
     <row r="527">

</xml_diff>